<commit_message>
Let MCP finish staged changes and give API keys a role.
confirm_action spends the same approval as Confirm. list_jobs defaults to
the workspace census. A workspace API key stores a role, and a key minted
before that field existed resolves to editor. Client snippets use the
absolute tenant MCP URL.

Co-authored-by: Venky-Chowdary <Venky-Chowdary@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/qe/DataFlow-QE-Test-Cases.xlsx
+++ b/docs/qe/DataFlow-QE-Test-Cases.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6">
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -581,27 +581,55 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>1. Dataset lookup. sample_payments and other underscore stems now bind the uploaded file. The word payment no longer selects the empty Financial Services template. Ambiguous column names stay unbound.</t>
+          <t>1. Dataset lookup binds the uploaded file. Production still returns the Financial Services template for sample_payments until deploy (TC-054).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2. Contract census. When the brief's contract page is full (50), the count comes from count_contracts_by_status, not from the page length. Production still reports 50 until this build is deployed. A fuller read already shows at least 200 contracts.</t>
+          <t>2. Contract census uses count_contracts_by_status when the brief page is full. list_contracts returns total, truncated, and by_status. Production still returns the page length until deploy.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Not changed: connector outages, the job-count gap between brief (workspace_id empty) and list_jobs (workspace_id omitted, all jobs), and no new transfer was written to PostgresVenkat.</t>
+          <t>3. list_jobs defaults to scope=workspace, the same population as the brief. scope=all is explicit. Production still returns 575 with no scope field (TC-040).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>4. confirm_action spends the same ack as Confirm. It is not on the deployed server (TC-051). A call with no request returns an error and does not mutate (TC-049).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>5. Workspace API keys store a role. A key with no role resolves to editor, so MCP can create connectors, transfers, and schedules. Unknown labels resolve to viewer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>6. MCP client snippets use the absolute tenant URL and a Bearer header. They do not point at api.datawrap.io or an unpublished bridge package.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Not changed: the 10 connector dial failures (TC-052), no schedule was created, and no new transfer was written to PostgresVenkat. CDC remains at-least-once upsert.</t>
         </is>
       </c>
     </row>
@@ -616,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2543,7 +2571,7 @@
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>brief 544 (failed 376, ok 162). list_jobs total 575</t>
+          <t>Live retest still shows brief 544 and list_jobs total 575 with no scope field. This build defaults list_jobs to scope=workspace (workspace_id ""), and scope=all is explicit.</t>
         </is>
       </c>
       <c r="H41" s="8" t="inlineStr">
@@ -2553,7 +2581,7 @@
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>list_jobs passes workspace_id None (all jobs). Brief passes "" (legacy/unscoped only). Not changed: picking either number would hide or widen tenant scope. Needs the caller workspace id on the MCP path.</t>
+          <t>Production has not deployed the scope parameter (retest 2026-10-04, total 575, keys count/jobs/status_counts/store/total). Unit test_job_list_scope.py passed: workspace -&gt; "", all -&gt; None.</t>
         </is>
       </c>
     </row>
@@ -2836,6 +2864,382 @@
       <c r="I47" s="6" t="inlineStr">
         <is>
           <t>The summary text is the honesty line. The per-cell status means the route is in the live matrix, not that this workspace just transferred it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>TC-047</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Jobs</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>services.job_list_scope</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>job_list_workspace_scope</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>workspace and this map to "". all maps to None. Any other token is refused.</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>15 pytest nodes in the operator set passed, including this function.</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>tests/test_job_list_scope.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>TC-048</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>API keys</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>services.api_key_role</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>resolve and parse role</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>A blank stored role is editor. An unknown label is viewer. owner is refused at create.</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>resolve(None|''|'  ')==editor. superuser==viewer. parse('owner') raises ValueError.</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>tests/test_api_key_role.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>TC-049</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>confirm_ack without a request</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>confirm_from_tool</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>ok false and no mutation</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Child process loaded the module without the agent runtime. ok is false. Error names ack_id or confirm_action.</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>tests/test_mcp_operator_scope.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>TC-050</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>mcpClientConfig</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>absolute URL and snippets</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://www.datawrap.io/api/v1/mcp with a Bearer placeholder. No api.datawrap.io. No mcp-bridge.</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>3 node tests passed.</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>apps/web/src/lib/mcpClientConfig.test.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>TC-051</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Live tools/list</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Look for confirm_action</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>The deployed server exposes confirm_action</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>51 tools. create_connector, start_transfer, and create_schedule are present. confirm_action is not, until this build is deployed.</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Live tools/list 2026-10-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>TC-052</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Connectors</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>11 saved connectors</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>test_connector on each</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Record the dial result. A refused host is not an engine defect.</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>1 pass: PostgresVenkat, 10 tables in public. 10 fail: Snowflake account/warehouse/database/schema/role (4), MySQL 2013 lost connection (4), Postgres server closed the connection, Redis connection reset.</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Live retest 2026-10-04. Same hosts as the first census. No connector was deleted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>TC-053</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Schedules</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Live workspace</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>list_schedules limit 50</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>The tool answers. An empty store stays empty.</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>ok, count 0, names []. No schedule was created or run.</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Live retest 2026-10-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>TC-054</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Datasets</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Live analyze_dataset sample_payments</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Name the upload, not the industry template</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>10-row sample_payments upload</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Production still returns Financial Services, row_count 0. scale_100k and sample_schema_types are still not found. sample_logistics returns the 5-row upload. The resolver fix is in this branch and is not deployed.</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Live retest 2026-10-04. 22 datasets listed, including the uploads.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stage uploaded files through the same confirm path as connector transfers.
start_dataset_transfer maps and preflights an upload, then stores a file ack.
Confirm keeps that kind and refuses a path outside the upload directory.

Co-authored-by: Venky-Chowdary <Venky-Chowdary@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/qe/DataFlow-QE-Test-Cases.xlsx
+++ b/docs/qe/DataFlow-QE-Test-Cases.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
@@ -630,6 +630,13 @@
       <c r="A16" t="inlineStr">
         <is>
           <t>Not changed: the 10 connector dial failures (TC-052), no schedule was created, and no new transfer was written to PostgresVenkat. CDC remains at-least-once upsert.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>7. start_dataset_transfer stages an uploaded file into a saved connector. Confirm keeps kind=file and refuses a path outside the upload directory. Measured on a payments.csv fixture, not on PostgresVenkat.</t>
         </is>
       </c>
     </row>
@@ -644,7 +651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3243,6 +3250,100 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>TC-055</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Transfers</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>services.confirmed_transfer</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Build a request from a confirm ack</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Database stays database. skip_preflight stays false. A file ack keeps kind=file and the upload path. A path outside the upload tree is refused.</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>4 tests passed, including /etc/passwd and an xfer_ spill.</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>tests/test_confirmed_transfer.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>TC-056</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Transfers</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>payments.csv fixture</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>start_dataset_transfer then read the ack</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Ack is start_transfer, source kind file, destination connector kept, mappings produced. A template name is refused. No rows written.</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2 tests passed. Preflight and dest introspect were the warehouse boundary; parse and mapping pipeline were real.</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>tests/test_dataset_transfer_stage.py</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Prove MCP confirm spends one connector, schedule, and file job.
confirm_action now runs through copilot_confirm against temporary stores:
one connector, one enabled schedule, one schedule run, and one file transfer
from sample_payments.csv. Replay returns the first result. A viewer refusal
and a path outside the upload tree leave the ack spendable.

Co-authored-by: Venky-Chowdary <Venky-Chowdary@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/qe/DataFlow-QE-Test-Cases.xlsx
+++ b/docs/qe/DataFlow-QE-Test-Cases.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
@@ -637,6 +637,13 @@
       <c r="A17" t="inlineStr">
         <is>
           <t>7. start_dataset_transfer stages an uploaded file into a saved connector. Confirm keeps kind=file and refuses a path outside the upload directory. Measured on a payments.csv fixture, not on PostgresVenkat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>8. confirm_action was run through copilot_confirm for a connector, an enabled schedule, a schedule run, and a file transfer. Replay returns the first result. A viewer refusal and a path outside the upload tree leave the ack spendable. 7 passed in tests/test_mcp_confirm_route.py. sample_payments.csv is the 10-row fixture. Nothing was written to PostgresVenkat.</t>
         </is>
       </c>
     </row>
@@ -651,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3344,6 +3351,335 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>TC-057</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Temporary connector file. test_first off.</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>create_connector then confirm_action as editor. Confirm the same ack again.</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>One connector is saved. Replay returns the same connector id and does not write a second row.</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>Passed. Name qe-mcp-confirm-connector, type postgresql. Store file was the test tmp path.</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_mcp_confirm_route.py::test_editor_confirm_saves_one_connector_and_replay_does_not_save_another</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>TC-058</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Viewer role, create_connector ack</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>confirm_action</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Refusal. The ack stays unconsumed. No connector row.</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>Passed. Error names the viewer role. peek consumed is false. Connector list empty.</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_mcp_confirm_route.py::test_viewer_confirm_of_create_connector_does_not_consume_the_ack</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>TC-059</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Schedules</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Mappings from run_mapping_pipeline for id, amount. Temporary schedules.json.</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>confirm_action on a create_schedule ack, then replay.</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>One enabled schedule. Cron kept. next_run_at set. Replay does not write a second schedule.</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>Passed. Name qe-mcp-nightly, cron 0 2 * * *, enabled true, one row in the temp store.</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_mcp_confirm_route.py::test_editor_confirm_creates_one_enabled_schedule_and_replay_keeps_one</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>TC-060</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Transfers</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>payments.csv under a temporary upload root. Engine call recorded.</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>confirm_action on a start_transfer ack with kind=file and skip_preflight true.</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>One engine request, kind=file, skip_preflight forced false. Replay does not call the engine again.</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>Passed. job-qe-file-1, source payments.csv, destination dest-qe.pay. Engine saw the request once.</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_mcp_confirm_route.py::test_file_ack_confirm_hands_the_upload_to_the_engine_once</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>TC-061</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Transfers</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>CSV sitting beside the upload root, not inside it.</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>confirm_action</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>Refusal. Engine is not called. Ack stays spendable.</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>Passed. Error says the file is outside the upload directory. peek consumed is false.</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_mcp_confirm_route.py::test_file_ack_outside_the_upload_tree_is_refused_and_stays_spendable</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>TC-062</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Transfers</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>tests/fixtures/sample_payments.csv (10 rows, CUST_ID through DESC)</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>start_dataset_transfer then confirm_action. Dest introspect and preflight are the warehouse boundary.</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>Preview rows 10. Confirm hands one kind=file request to the engine, path is the fixture, mappings include CUST_ID and AMT. Replay returns the same job.</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>Passed. job-payments-1, destination dest-qe.payments_wh. Parse and mapping pipeline were real. No warehouse write.</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_mcp_confirm_route.py::test_staged_payments_file_confirms_into_one_engine_request</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>TC-063</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Schedules</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>Enabled schedule in a temporary file. Runner call recorded.</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>confirm_action on a run_schedule ack, then replay.</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>Runner called once with manual true. Replay returns the same job id and does not call again.</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>Passed. job-schedule-1. The real runner was not asked to dial a connector.</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_mcp_confirm_route.py::test_confirm_runs_a_schedule_once</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Let MCP create a SQLite file and load a real CSV into it.
A SQLite or DuckDB connector is a path, so the draft no longer demands a
host. The probe uses the same path allowlist as the reader. Streamable MCP
then loads the 10-row payments fixture into that file and a schedule copies
it into a second SQLite file. Both counts stay 10 on replay.

Co-authored-by: Venky-Chowdary <Venky-Chowdary@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/qe/DataFlow-QE-Test-Cases.xlsx
+++ b/docs/qe/DataFlow-QE-Test-Cases.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
@@ -644,6 +644,13 @@
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>8. confirm_action was run through copilot_confirm for a connector, an enabled schedule, a schedule run, and a file transfer. Replay returns the first result. A viewer refusal and a path outside the upload tree leave the ack spendable. 7 passed in tests/test_mcp_confirm_route.py. sample_payments.csv is the 10-row fixture. Nothing was written to PostgresVenkat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>9. MCP can create a SQLite connector from a file path. Streamable POST /api/v1/mcp loaded sample_payments.csv (10 rows) into that file, scheduled the table onto a second SQLite file, and ran the schedule. Both tables counted 10. Replay did not insert again. tests/test_mcp_sqlite_file_transfer.py passed. The probe and the draft share sqlite_file_path.</t>
         </is>
       </c>
     </row>
@@ -658,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3680,6 +3687,100 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>TC-064</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Connectors</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>SQLite file under DATAFLOW_SQLITE_ROOT. No host, no password.</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>draft_is_complete and test_sqlite</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>A path inside the root is complete and the probe opens it. A path outside the root is refused by both. DuckDB is complete with a file path. Postgres without a host is refused.</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>Passed. tests/test_pilot_create_connector.py, two new cases, 6 passed in that file.</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_pilot_create_connector.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>TC-065</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>tests/fixtures/sample_payments.csv (10 rows) via POST /api/v1/mcp</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>create_connector sqlite, confirm, start_dataset_transfer, confirm, create_schedule onto a second sqlite file, confirm, run_schedule_now, confirm, replay</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>payments COUNT is 10. payments_wh COUNT is 10. Replay does not insert again.</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>Passed in 1 test. Streamable MCP, real preflight, real engine, real schedule runner. Both sqlite files were under a temporary SQLITE_ROOT. No write to PostgresVenkat.</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t>tests/test_mcp_sqlite_file_transfer.py::test_mcp_loads_sample_payments_into_sqlite</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Let MCP load typed files and declare a timestamp zone.
File columns the parser did not type are no longer treated as declared TEXT, so JSONL timestamps and binary values stamp SQLite TIMESTAMPTZ and BLOB. A column that mixes wall-clock values with offsets stays blocked until source_timezone names an IANA zone. The streamable MCP proof loads a TSV, a JSON array, and that JSONL, then pauses and deletes the schedule.

Co-authored-by: Venky-Chowdary <Venky-Chowdary@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/qe/DataFlow-QE-Test-Cases.xlsx
+++ b/docs/qe/DataFlow-QE-Test-Cases.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
@@ -651,6 +651,13 @@
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>9. MCP can create a SQLite connector from a file path. Streamable POST /api/v1/mcp loaded sample_payments.csv (10 rows) into that file, scheduled the table onto a second SQLite file, and ran the schedule. Both tables counted 10. Replay did not insert again. tests/test_mcp_sqlite_file_transfer.py passed. The probe and the draft share sqlite_file_path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10. File columns the parser did not type are not declared TEXT. JSONL sample_mixed_types is refused until source_timezone is an IANA zone, then loads 3 rows into SQLite with created_at TIMESTAMPTZ and payload_b64 BLOB. TSV is 3 rows, HR JSON is 5. The HR schedule pauses and deletes through confirm_action. tests/test_mcp_sqlite_file_transfer.py: 2 passed. Nothing was written to PostgresVenkat.</t>
         </is>
       </c>
     </row>
@@ -665,7 +672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3781,6 +3788,147 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>TC-066</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>tests/fixtures/sample_mixed_types.jsonl (3 rows, mixed offsets)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>start_dataset_transfer with no source_timezone, then with source_timezone=Not/AZone</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Both calls are refused. The first names created_at and naive wall-clock and tells the operator to pass source_timezone. The second names the unknown zone. No mixed table is created.</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Passed. Refusal happened before confirm, so the engine did not write.</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>tests/test_mcp_sqlite_file_transfer.py::test_mcp_loads_tsv_json_and_jsonl_then_pauses_and_deletes_the_schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>TC-067</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Transfers</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>sample_payments.tsv (3), sample_hr.json (5), sample_mixed_types.jsonl with source_timezone=UTC</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>start_dataset_transfer and confirm for each file into one SQLite connector</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>payments_tsv COUNT 3 and CUST_ID 2001. hr COUNT 5 and emp_id E001. mixed COUNT 3, metadata_json contains us-east, created_at DDL is TIMESTAMPTZ with clocks 12:00:00, 15:30:00, 08:00:00, payload_b64 is BLOB.</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Passed. Streamable MCP, real preflight, real engine. SQLite files were under a temporary SQLITE_ROOT.</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>tests/test_mcp_sqlite_file_transfer.py::test_mcp_loads_tsv_json_and_jsonl_then_pauses_and_deletes_the_schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>TC-068</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Schedules</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Schedule qe-mcp-hr-nightly from hr to a second SQLite file</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>create_schedule, confirm, set_schedule_enabled false, confirm, delete_schedule, confirm, list_schedules</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>The schedule is enabled, then paused, then gone. list_schedules count is 0.</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Passed. Confirm ran each step once against the isolated schedule store.</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>tests/test_mcp_sqlite_file_transfer.py::test_mcp_loads_tsv_json_and_jsonl_then_pauses_and_deletes_the_schedule</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Let MCP change a pipeline cadence without re-planning the route.
update_schedule stages interval, cron, and timezone on the existing schedule
patch. An hourly cadence clears a previous cron. A file load into a SQLite
table whose columns are reversed still writes CUST_ID by name.

Co-authored-by: Venky-Chowdary <Venky-Chowdary@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/qe/DataFlow-QE-Test-Cases.xlsx
+++ b/docs/qe/DataFlow-QE-Test-Cases.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
@@ -658,6 +658,13 @@
       <c r="A20" t="inlineStr">
         <is>
           <t>10. File columns the parser did not type are not declared TEXT. JSONL sample_mixed_types is refused until source_timezone is an IANA zone, then loads 3 rows into SQLite with created_at TIMESTAMPTZ and payload_b64 BLOB. TSV is 3 rows, HR JSON is 5. The HR schedule pauses and deletes through confirm_action. tests/test_mcp_sqlite_file_transfer.py: 2 passed. Nothing was written to PostgresVenkat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>11. MCP update_schedule changes a pipeline cadence through the existing schedule PATCH. qe-mcp-payments-nightly moved from cron 0 2 * * * to 0 3 * * * and then to hourly with the cron cleared. The schedule id, enabled flag, route, and mappings stayed. Replay did not apply the clock twice. A file load into an existing SQLite table with columns in reverse CSV order kept CUST_ID 1001 and DESC containing Wire. tests/test_mcp_sqlite_file_transfer.py: 3 passed. tests/test_pilot_lifecycle_tools.py: 59 passed. Nothing was written to PostgresVenkat.</t>
         </is>
       </c>
     </row>
@@ -672,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3929,6 +3936,100 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>TC-069</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Schedules</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>qe-mcp-payments-nightly, daily at 02:00 UTC, after the 10-row SQLite load</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>update_schedule to the same cadence, to whenever, to daily at 03:00 UTC, confirm, replay, then hourly, confirm. Read the stored schedule.</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Same cadence and an unresolved phrase are refused. Confirm keeps the schedule id and enabled flag, sets cron 0 3 * * *, and does not replace mappings. Replay does not move the clock. Hourly clears cron.</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Passed. Streamable MCP against the isolated schedule store. Mappings after both confirms equalled the mappings saved at create. Nothing was written to PostgresVenkat.</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>tests/test_mcp_sqlite_file_transfer.py::test_mcp_loads_sample_payments_into_sqlite</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>TC-070</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Transfers</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>sample_payments.csv into SQLite table landed. Columns reversed: DESC, STS, REF_NO, CCY, ACCT_NO, TXN_DT DATE, AMT DECIMAL(8,2), CUST_ID BIGINT.</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>create_connector, create the table, start_dataset_transfer full_refresh_append, confirm.</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>PRAGMA order stays DESC first and CUST_ID last. COUNT 10. CUST_ID 1001. DESC contains Wire. AMT 1500.</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Passed. Dest-exists write used the existing table. Positional jumble would have put the description in CUST_ID.</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>tests/test_mcp_sqlite_file_transfer.py::test_mcp_file_load_into_existing_sqlite_writes_by_column_name</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>